<commit_message>
Actualizacion datos REM 2026-09-29 16:28 (orquestador)
</commit_message>
<xml_diff>
--- a/comparacion.xlsx
+++ b/comparacion.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="70">
   <si>
     <t>Indicador</t>
   </si>
@@ -88,27 +88,15 @@
     <t>Proxy</t>
   </si>
   <si>
-    <t>58,04%</t>
-  </si>
-  <si>
     <t>64,50%</t>
   </si>
   <si>
-    <t>37,43%</t>
-  </si>
-  <si>
     <t>4,36%</t>
   </si>
   <si>
-    <t>63,30%</t>
-  </si>
-  <si>
     <t>44,54%</t>
   </si>
   <si>
-    <t>28,19%</t>
-  </si>
-  <si>
     <t>19,26%</t>
   </si>
   <si>
@@ -205,10 +193,7 @@
     <t>50.413</t>
   </si>
   <si>
-    <t>1.272.273</t>
-  </si>
-  <si>
-    <t>566.991</t>
+    <t>0</t>
   </si>
   <si>
     <t>108.051</t>
@@ -217,19 +202,7 @@
     <t>95.604</t>
   </si>
   <si>
-    <t>+0,017 pp</t>
-  </si>
-  <si>
-    <t>+0,056 pp</t>
-  </si>
-  <si>
     <t>-0,027 pp</t>
-  </si>
-  <si>
-    <t>+0,705 pp</t>
-  </si>
-  <si>
-    <t>+0,308 pp</t>
   </si>
   <si>
     <t>-0,025 pp</t>
@@ -615,20 +588,14 @@
       <c r="B2" t="s">
         <v>22</v>
       </c>
-      <c r="C2" t="s">
-        <v>24</v>
-      </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F2" t="s">
-        <v>63</v>
-      </c>
-      <c r="G2" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -639,13 +606,13 @@
         <v>22</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F3" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -655,20 +622,14 @@
       <c r="B4" t="s">
         <v>22</v>
       </c>
-      <c r="C4" t="s">
-        <v>26</v>
-      </c>
       <c r="D4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F4" t="s">
-        <v>63</v>
-      </c>
-      <c r="G4" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -679,19 +640,19 @@
         <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F5" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G5" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -701,20 +662,14 @@
       <c r="B6" t="s">
         <v>22</v>
       </c>
-      <c r="C6" t="s">
-        <v>28</v>
-      </c>
       <c r="D6" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E6" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F6" t="s">
-        <v>64</v>
-      </c>
-      <c r="G6" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -725,13 +680,13 @@
         <v>22</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -741,20 +696,14 @@
       <c r="B8" t="s">
         <v>22</v>
       </c>
-      <c r="C8" t="s">
-        <v>30</v>
-      </c>
       <c r="D8" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E8" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F8" t="s">
-        <v>64</v>
-      </c>
-      <c r="G8" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -765,19 +714,19 @@
         <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D9" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="E9" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F9" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G9" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -788,19 +737,19 @@
         <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D10" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E10" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F10" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G10" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -811,19 +760,19 @@
         <v>22</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E11" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F11" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G11" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -834,13 +783,13 @@
         <v>22</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E12" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F12" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -851,19 +800,19 @@
         <v>22</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D13" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" t="s">
+        <v>55</v>
+      </c>
+      <c r="F13" t="s">
         <v>46</v>
       </c>
-      <c r="E13" t="s">
-        <v>59</v>
-      </c>
-      <c r="F13" t="s">
-        <v>50</v>
-      </c>
       <c r="G13" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -874,19 +823,19 @@
         <v>22</v>
       </c>
       <c r="C14" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D14" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E14" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F14" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G14" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -897,19 +846,19 @@
         <v>23</v>
       </c>
       <c r="C15" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D15" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E15" t="s">
+        <v>57</v>
+      </c>
+      <c r="F15" t="s">
         <v>61</v>
       </c>
-      <c r="F15" t="s">
-        <v>66</v>
-      </c>
       <c r="G15" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -920,19 +869,19 @@
         <v>23</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D16" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E16" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F16" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="G16" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: coberturas PIV 1,3,6,8 (es_aps Primer Nivel + join por IDs), egresos F->G, config_rutas, legacy D congelado
</commit_message>
<xml_diff>
--- a/comparacion.xlsx
+++ b/comparacion.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="79">
   <si>
     <t>Indicador</t>
   </si>
@@ -88,15 +88,27 @@
     <t>Proxy</t>
   </si>
   <si>
+    <t>57,82%</t>
+  </si>
+  <si>
     <t>64,50%</t>
   </si>
   <si>
+    <t>37,30%</t>
+  </si>
+  <si>
     <t>4,36%</t>
   </si>
   <si>
+    <t>63,06%</t>
+  </si>
+  <si>
     <t>44,54%</t>
   </si>
   <si>
+    <t>28,09%</t>
+  </si>
+  <si>
     <t>19,26%</t>
   </si>
   <si>
@@ -193,7 +205,10 @@
     <t>50.413</t>
   </si>
   <si>
-    <t>0</t>
+    <t>1.276.928</t>
+  </si>
+  <si>
+    <t>569.066</t>
   </si>
   <si>
     <t>108.051</t>
@@ -202,7 +217,19 @@
     <t>95.604</t>
   </si>
   <si>
+    <t>-0,195 pp</t>
+  </si>
+  <si>
+    <t>-0,080 pp</t>
+  </si>
+  <si>
     <t>-0,027 pp</t>
+  </si>
+  <si>
+    <t>+0,474 pp</t>
+  </si>
+  <si>
+    <t>+0,205 pp</t>
   </si>
   <si>
     <t>-0,025 pp</t>
@@ -588,14 +615,20 @@
       <c r="B2" t="s">
         <v>22</v>
       </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F2" t="s">
-        <v>59</v>
+        <v>63</v>
+      </c>
+      <c r="G2" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -606,13 +639,13 @@
         <v>22</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F3" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -622,14 +655,20 @@
       <c r="B4" t="s">
         <v>22</v>
       </c>
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
       <c r="D4" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F4" t="s">
-        <v>59</v>
+        <v>63</v>
+      </c>
+      <c r="G4" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -640,19 +679,19 @@
         <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E5" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G5" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -662,14 +701,20 @@
       <c r="B6" t="s">
         <v>22</v>
       </c>
+      <c r="C6" t="s">
+        <v>28</v>
+      </c>
       <c r="D6" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="E6" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F6" t="s">
-        <v>59</v>
+        <v>64</v>
+      </c>
+      <c r="G6" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -680,13 +725,13 @@
         <v>22</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E7" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="F7" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -696,14 +741,20 @@
       <c r="B8" t="s">
         <v>22</v>
       </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
       <c r="D8" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E8" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="F8" t="s">
-        <v>59</v>
+        <v>64</v>
+      </c>
+      <c r="G8" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -714,19 +765,19 @@
         <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E9" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F9" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G9" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -737,19 +788,19 @@
         <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D10" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E10" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F10" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="G10" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -760,19 +811,19 @@
         <v>22</v>
       </c>
       <c r="C11" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D11" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E11" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11" t="s">
         <v>53</v>
       </c>
-      <c r="F11" t="s">
-        <v>49</v>
-      </c>
       <c r="G11" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -783,13 +834,13 @@
         <v>22</v>
       </c>
       <c r="C12" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E12" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F12" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -800,19 +851,19 @@
         <v>22</v>
       </c>
       <c r="C13" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D13" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E13" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F13" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G13" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -823,19 +874,19 @@
         <v>22</v>
       </c>
       <c r="C14" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E14" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F14" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G14" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -846,19 +897,19 @@
         <v>23</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D15" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E15" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F15" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G15" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -869,19 +920,19 @@
         <v>23</v>
       </c>
       <c r="C16" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D16" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E16" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="F16" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G16" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>